<commit_message>
Adiciona painel admin e registro em lote
</commit_message>
<xml_diff>
--- a/relatorio_refeicoes.xlsx
+++ b/relatorio_refeicoes.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,35 +468,72 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>15/01/2026</t>
+          <t>18/01/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>20:37</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>samuel</t>
+          <t>Timotio</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>177</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Alfa</t>
+          <t>a</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Dono</t>
+          <t>a</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
+        <is>
+          <t>Café da Manhã</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>18/01/2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Betina</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>Almoço</t>
         </is>

</xml_diff>